<commit_message>
data: update 2026-09-09 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>8</v>
@@ -883,7 +883,7 @@
         <v>41</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.78</v>
+        <v>4.8</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-13</v>
+        <v>-8</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.24</v>
+        <v>5.25</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.37</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=-5.0bp
-HYG 5d=-0.2% [OK]
+          <t>HY OAS 20dd=5.0bp [OK]
+HY OAS 5dd=-2.0bp
+HYG 5d=-0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=2.5% [OK]
-SPY vs 200MA: above ($SPY=770.1900024414062, 200MA=709.9)
+FXY 5d=3.8% [TRIGGERED]
+SPY vs 200MA: above ($SPY=765.9600219726562, 200MA=710.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-10 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>45</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.43</v>
+        <v>2.46</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.8</v>
+        <v>4.83</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-8</v>
+        <v>-13</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.25</v>
+        <v>5.28</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-10</v>
+        <v>-14</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.64</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2894.53</v>
+        <v>2991.31</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>235.06</v>
+        <v>-89.48</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.71</v>
+        <v>6.76</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-41</v>
+        <v>-53</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=5.0bp [OK]
-HY OAS 5dd=-2.0bp
-HYG 5d=-0.3% [OK]
+          <t>HY OAS 20dd=0.0bp [OK]
+HY OAS 5dd=-5.0bp
+HYG 5d=-0.2% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=3.8% [TRIGGERED]
-SPY vs 200MA: above ($SPY=765.9600219726562, 200MA=710.4)
+FXY 5d=4.4% [TRIGGERED]
+SPY vs 200MA: above ($SPY=762.4000244140625, 200MA=711.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-11 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.46</v>
+        <v>2.55</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-3</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.83</v>
+        <v>4.95</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-13</v>
+        <v>-27</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.28</v>
+        <v>5.37</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-4</v>
+        <v>-13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.4</v>
+        <v>2.36</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>0</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>0</v>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=0.0bp [OK]
+          <t>HY OAS 20dd=1.0bp [OK]
 HY OAS 5dd=-5.0bp
-HYG 5d=-0.2% [OK]
+HYG 5d=-0.6% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=4.4% [TRIGGERED]
-SPY vs 200MA: above ($SPY=762.4000244140625, 200MA=711.0)
+FXY 5d=2.9% [TRIGGERED]
+SPY vs 200MA: above ($SPY=757.8300170898438, 200MA=711.5)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-15 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>-21</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-27</v>
+        <v>-33</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.37</v>
+        <v>5.35</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=1.0bp [OK]
-HY OAS 5dd=-5.0bp
-HYG 5d=-0.6% [OK]
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=2.9% [TRIGGERED]
-SPY vs 200MA: above ($SPY=757.8300170898438, 200MA=711.5)
+FXY 5d=nan% [OK]
+SPY vs 200MA: above ($SPY=nan, 200MA=nan)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-16 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.6</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-21</v>
+        <v>-19</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.96</v>
+        <v>4.97</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-33</v>
+        <v>-29</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.35</v>
+        <v>5.34</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-14</v>
+        <v>-9</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.37</v>
+        <v>2.38</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-10</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>-4</v>
@@ -1984,7 +1984,7 @@
         <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=3.0bp
+          <t>HY OAS 20dd=-1.0bp [OK]
+HY OAS 5dd=-3.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-09-18 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>27</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.68</v>
+        <v>2.61</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.01</v>
+        <v>4.94</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.35</v>
+        <v>5.29</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-28</v>
+        <v>-5</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>-27</v>
+        <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.62</v>
+        <v>3.85</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>3</v>
+        <v>-23</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>8</v>
+        <v>-11</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=3.0bp [OK]
-HY OAS 5dd=1.0bp
-HYG 5d=-0.7% [OK]
+          <t>HY OAS 20dd=5.0bp [OK]
+HY OAS 5dd=0.0bp
+HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.6% [OK]
-SPY vs 200MA: above ($SPY=754.0499877929688, 200MA=713.4)
+FXY 5d=-1.1% [OK]
+SPY vs 200MA: above ($SPY=762.5999755859375, 200MA=713.8)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-22 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46283</v>
+        <v>46287</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.61</v>
+        <v>2.68</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-26</v>
+        <v>-33</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.94</v>
+        <v>5.01</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-29</v>
+        <v>-32</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.29</v>
+        <v>5.34</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1624,7 +1624,7 @@
         <v>-5</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.85</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>4</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=5.0bp [OK]
-HY OAS 5dd=0.0bp
-HYG 5d=0.1% [OK]
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=-3.0bp
+HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-1.1% [OK]
-SPY vs 200MA: above ($SPY=762.5999755859375, 200MA=713.8)
+FXY 5d=nan% [OK]
+SPY vs 200MA: above ($SPY=nan, 200MA=nan)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-23 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.68</v>
+        <v>2.62</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-33</v>
+        <v>-22</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.01</v>
+        <v>4.96</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-32</v>
+        <v>-22</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.34</v>
+        <v>5.29</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-11</v>
+        <v>-2</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.34</v>
+        <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-5</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-3</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.85</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-22</v>
+        <v>-20</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>5</v>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=-3.0bp
+          <t>HY OAS 20dd=3.0bp [OK]
+HY OAS 5dd=5.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-09-24 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>46</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>13</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.62</v>
+        <v>2.63</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-22</v>
+        <v>-25</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1067,7 +1067,7 @@
         <v>4.96</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-22</v>
+        <v>-26</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1096,7 +1096,7 @@
         <v>5.29</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.33</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.36</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.85</v>
+        <v>3.87</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-20</v>
+        <v>-22</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
         <v>135</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=3.0bp [OK]
-HY OAS 5dd=5.0bp
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=8.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-09-25 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F13" s="24" t="n">
         <v>21</v>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.63</v>
+        <v>2.76</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-25</v>
+        <v>-44</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.96</v>
+        <v>5.11</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-26</v>
+        <v>-47</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.29</v>
+        <v>5.4</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-6</v>
+        <v>-23</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.36</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.87</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3013.79</v>
+        <v>2930.19</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-95.19</v>
+        <v>102.39</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>77</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>2</v>
+        <v>-6</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.95</v>
+        <v>7.03</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-65</v>
+        <v>-66</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=2.0bp [OK]
-HY OAS 5dd=8.0bp
+          <t>HY OAS 20dd=-6.0bp [OK]
+HY OAS 5dd=-3.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-09-26 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>29</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.76</v>
+        <v>2.85</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-44</v>
+        <v>-51</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.11</v>
+        <v>5.18</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-47</v>
+        <v>-52</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.4</v>
+        <v>5.47</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-23</v>
+        <v>-29</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-1</v>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.87</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-21</v>
+        <v>-24</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-6</v>
+        <v>-17</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-6.0bp [OK]
-HY OAS 5dd=-3.0bp
+          <t>HY OAS 20dd=-17.0bp [OK]
+HY OAS 5dd=-10.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-09-29 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46291</v>
+        <v>46294</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.85</v>
+        <v>2.83</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-51</v>
+        <v>-49</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-52</v>
+        <v>-50</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.47</v>
+        <v>5.49</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-24</v>
+        <v>-26</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-17</v>
+        <v>-33</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>5</v>
+        <v>-4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-17.0bp [OK]
-HY OAS 5dd=-10.0bp
-HYG 5d=nan% [OK]
+          <t>HY OAS 20dd=-33.0bp [OK]
+HY OAS 5dd=-25.0bp
+HYG 5d=-1.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=nan% [OK]
-SPY vs 200MA: above ($SPY=nan, 200MA=nan)
+FXY 5d=0.0% [OK]
+SPY vs 200MA: above ($SPY=765.6099853515625, 200MA=715.3)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-09-30 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>32</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.83</v>
+        <v>2.9</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-49</v>
+        <v>-48</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.17</v>
+        <v>5.24</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-50</v>
+        <v>-51</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.49</v>
+        <v>5.56</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-30</v>
+        <v>-34</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.9</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-33</v>
+        <v>-39</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-33.0bp [OK]
-HY OAS 5dd=-25.0bp
-HYG 5d=-1.4% [OK]
+          <t>HY OAS 20dd=-39.0bp [OK]
+HY OAS 5dd=-36.0bp
+HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.0% [OK]
-SPY vs 200MA: above ($SPY=765.6099853515625, 200MA=715.3)
+FXY 5d=nan% [OK]
+SPY vs 200MA: above ($SPY=nan, 200MA=nan)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-01 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>17</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.9</v>
+        <v>2.91</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-48</v>
+        <v>-47</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.24</v>
+        <v>5.26</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-51</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.56</v>
+        <v>5.59</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-34</v>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.36</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.9</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-25</v>
+        <v>-20</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-3</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-39</v>
+        <v>-43</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-39.0bp [OK]
-HY OAS 5dd=-36.0bp
+          <t>HY OAS 20dd=-43.0bp [OK]
+HY OAS 5dd=-40.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-02 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Steepening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>20</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.91</v>
+        <v>2.93</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-47</v>
+        <v>-49</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.26</v>
+        <v>5.29</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-51</v>
+        <v>-50</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.59</v>
+        <v>5.64</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-34</v>
+        <v>-37</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.36</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-20</v>
+        <v>-24</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2930.19</v>
+        <v>2948.09</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>102.39</v>
+        <v>154.72</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-43</v>
+        <v>-46</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-11</v>
+        <v>-13</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>7.03</v>
+        <v>7.28</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-66</v>
+        <v>-92</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-43.0bp [OK]
-HY OAS 5dd=-40.0bp
+          <t>HY OAS 20dd=-46.0bp [OK]
+HY OAS 5dd=-39.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-03 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-1</v>
+        <v>-6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.93</v>
+        <v>2.88</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-49</v>
+        <v>-43</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.29</v>
+        <v>5.24</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-50</v>
+        <v>-45</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.64</v>
+        <v>5.61</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-37</v>
+        <v>-34</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.36</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.9</v>
+        <v>3.87</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-24</v>
+        <v>-22</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-46</v>
+        <v>-59</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-13</v>
+        <v>-23</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>11</v>
+        <v>-15</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-46.0bp [OK]
-HY OAS 5dd=-39.0bp
+          <t>HY OAS 20dd=-59.0bp [OK]
+HY OAS 5dd=-44.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-06 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Bull Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.88</v>
+        <v>2.92</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-43</v>
+        <v>-50</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.24</v>
+        <v>5.28</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-45</v>
+        <v>-51</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.61</v>
+        <v>5.63</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-34</v>
+        <v>-38</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
         <v>3</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
         <v>3</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.87</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-22</v>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-59</v>
+        <v>-42</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-59.0bp [OK]
-HY OAS 5dd=-44.0bp
-HYG 5d=nan% [OK]
+          <t>HY OAS 20dd=-42.0bp [OK]
+HY OAS 5dd=-17.0bp
+HYG 5d=-0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=nan% [OK]
-SPY vs 200MA: above ($SPY=nan, 200MA=nan)
+FXY 5d=-0.3% [OK]
+SPY vs 200MA: above ($SPY=774.8300170898438, 200MA=717.6)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-07 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>35</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.92</v>
+        <v>2.95</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-50</v>
+        <v>-52</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.28</v>
+        <v>5.31</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-51</v>
+        <v>-53</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.63</v>
+        <v>5.66</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-38</v>
+        <v>-42</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.36</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>3</v>
+        <v>-24</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>0</v>
+        <v>-25</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1746,7 +1746,7 @@
         <v>3.9</v>
       </c>
       <c r="F42" s="24" t="n">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="G42" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.89</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-42</v>
+        <v>-44</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-42.0bp [OK]
-HY OAS 5dd=-17.0bp
-HYG 5d=-0.3% [OK]
+          <t>HY OAS 20dd=-44.0bp [OK]
+HY OAS 5dd=-10.0bp
+HYG 5d=0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.3% [OK]
-SPY vs 200MA: above ($SPY=774.8300170898438, 200MA=717.6)
+FXY 5d=-0.6% [OK]
+SPY vs 200MA: above ($SPY=779.0900268554688, 200MA=718.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-08 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-1</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.95</v>
+        <v>2.91</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-52</v>
+        <v>-48</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.31</v>
+        <v>5.27</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-53</v>
+        <v>-47</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.66</v>
+        <v>5.64</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-42</v>
+        <v>-39</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1436,7 +1436,7 @@
         <v>2.35</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-24</v>
+        <v>-26</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.89</v>
+        <v>3.9</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-24</v>
+        <v>-26</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-44</v>
+        <v>-36</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-21</v>
+        <v>-19</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-44.0bp [OK]
-HY OAS 5dd=-10.0bp
-HYG 5d=0.3% [OK]
+          <t>HY OAS 20dd=-36.0bp [OK]
+HY OAS 5dd=5.0bp
+HYG 5d=0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.6% [OK]
-SPY vs 200MA: above ($SPY=779.0900268554688, 200MA=718.1)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=777.219970703125, 200MA=718.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-09 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-48</v>
+        <v>-46</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.27</v>
+        <v>5.28</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-47</v>
+        <v>-45</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.64</v>
+        <v>5.67</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-39</v>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.9</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2948.09</v>
+        <v>3029.66</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>154.72</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-36</v>
+        <v>-38</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>7.28</v>
+        <v>7.4</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-92</v>
+        <v>-89</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-36.0bp [OK]
-HY OAS 5dd=5.0bp
-HYG 5d=0.4% [OK]
+          <t>HY OAS 20dd=-38.0bp [OK]
+HY OAS 5dd=3.0bp
+HYG 5d=0.3% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=777.219970703125, 200MA=718.7)
+FXY 5d=0.1% [OK]
+SPY vs 200MA: above ($SPY=773.9299926757812, 200MA=719.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-10 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-3</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.92</v>
+        <v>2.87</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-46</v>
+        <v>-32</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.28</v>
+        <v>5.22</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-45</v>
+        <v>-27</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.67</v>
+        <v>5.6</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-39</v>
+        <v>-23</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F40" s="24" t="n">
         <v>0</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <v>1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.87</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-24</v>
+        <v>-25</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1984,7 +1984,7 @@
         <v>82</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-38</v>
+        <v>-45</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-21</v>
+        <v>-27</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-15</v>
+        <v>-24</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-38.0bp [OK]
-HY OAS 5dd=3.0bp
-HYG 5d=0.3% [OK]
+          <t>HY OAS 20dd=-45.0bp [OK]
+HY OAS 5dd=9.0bp
+HYG 5d=0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.1% [OK]
-SPY vs 200MA: above ($SPY=773.9299926757812, 200MA=719.2)
+FXY 5d=-0.3% [OK]
+SPY vs 200MA: above ($SPY=778.5700073242188, 200MA=719.7)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-13 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -2918,8 +2918,8 @@
 HY OAS 5dd=9.0bp
 HYG 5d=0.4% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.3% [OK]
-SPY vs 200MA: above ($SPY=778.5700073242188, 200MA=719.7)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=778.0999755859375, 200MA=720.1)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-14 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-8</v>
+        <v>-11</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.87</v>
+        <v>2.91</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.22</v>
+        <v>5.24</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1096,7 +1096,7 @@
         <v>5.6</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-23</v>
+        <v>-25</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.33</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.32</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-45</v>
+        <v>-40</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-27</v>
+        <v>-20</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-45.0bp [OK]
-HY OAS 5dd=9.0bp
-HYG 5d=0.4% [OK]
+          <t>HY OAS 20dd=-40.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.4% [OK]
-SPY vs 200MA: above ($SPY=778.0999755859375, 200MA=720.1)
+FXY 5d=nan% [OK]
+SPY vs 200MA: above ($SPY=nan, 200MA=nan)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-15 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F15" s="24" t="n">
         <v>-8</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-4</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.91</v>
+        <v>2.88</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-31</v>
+        <v>-28</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.24</v>
+        <v>5.21</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-28</v>
+        <v>-24</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.6</v>
+        <v>5.56</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-25</v>
+        <v>-22</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.33</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>1</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-25</v>
+        <v>-27</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.87</v>
+        <v>3.89</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-25</v>
+        <v>-27</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>-40</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-20</v>
+        <v>-17</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-40.0bp [OK]
-HY OAS 5dd=1.0bp
+HY OAS 5dd=-13.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-16 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-8</v>
+        <v>-1</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.88</v>
+        <v>2.84</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-28</v>
+        <v>-22</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.21</v>
+        <v>5.19</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-24</v>
+        <v>-19</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.56</v>
+        <v>5.52</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-22</v>
+        <v>-16</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.32</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.34</v>
+        <v>2.31</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-27</v>
+        <v>-24</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="24" t="n">
         <v>1</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.89</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-27</v>
+        <v>-24</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3029.66</v>
+        <v>3022.14</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>99.90000000000001</v>
+        <v>44.42</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-40</v>
+        <v>-55</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-17</v>
+        <v>-22</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2474,7 +2474,7 @@
         <v>7.4</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-89</v>
+        <v>-87</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-40.0bp [OK]
-HY OAS 5dd=-13.0bp
+          <t>HY OAS 20dd=-55.0bp [OK]
+HY OAS 5dd=-16.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-17 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>19</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.84</v>
+        <v>2.78</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-22</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.19</v>
+        <v>5.1</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-19</v>
+        <v>-9</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.52</v>
+        <v>5.43</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-16</v>
+        <v>-8</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.32</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-24</v>
+        <v>-27</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.89</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-24</v>
+        <v>-27</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-55</v>
+        <v>-53</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>-22</v>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-24</v>
+        <v>-22</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-55.0bp [OK]
-HY OAS 5dd=-16.0bp
+          <t>HY OAS 20dd=-53.0bp [OK]
+HY OAS 5dd=-8.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-20 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>-3</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>1</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Flattening</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>-4</v>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.78</v>
+        <v>2.74</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-10</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.1</v>
+        <v>5.09</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1096,7 +1096,7 @@
         <v>5.43</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-8</v>
+        <v>-14</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.32</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-27</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.89</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-27</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-53</v>
+        <v>-63</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-22</v>
+        <v>-27</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-53.0bp [OK]
-HY OAS 5dd=-8.0bp
+          <t>HY OAS 20dd=-63.0bp [OK]
+HY OAS 5dd=-20.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-21 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>54</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-8</v>
+        <v>-13</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-7</v>
+        <v>-13</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.74</v>
+        <v>2.8</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.09</v>
+        <v>5.15</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.43</v>
+        <v>5.48</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-14</v>
@@ -1353,7 +1353,7 @@
         <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.32</v>
+        <v>2.31</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F38" s="24" t="n">
         <v>-2</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.87</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>-63</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-27</v>
+        <v>-25</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2915,7 +2915,7 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-63.0bp [OK]
-HY OAS 5dd=-20.0bp
+HY OAS 5dd=-18.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-22 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Flattening</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>-12</v>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.15</v>
+        <v>0</v>
       </c>
       <c r="F19" s="24" t="n">
         <v>-14</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.48</v>
+        <v>0</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>-14</v>
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>0</v>
       </c>
       <c r="F29" s="24" t="n">
         <v>-1</v>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>4</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F39" s="24" t="n">
         <v>0</v>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="E42" s="24" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="F42" s="24" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.87</v>
+        <v>0</v>
       </c>
       <c r="F43" s="24" t="n">
         <v>-2</v>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>3022.14</v>
+        <v>0</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>44.42</v>
+        <v>0</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="F66" s="24" t="n">
         <v>-87</v>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-63.0bp [OK]
-HY OAS 5dd=-18.0bp
+          <t>HY OAS 20dd=Nonebp [OK]
+HY OAS 5dd=Nonebp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-23 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-13</v>
+        <v>-7</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bull Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-13</v>
+        <v>-3</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>0</v>
+        <v>2.76</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>0</v>
+        <v>5.13</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-14</v>
+        <v>-17</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>0</v>
+        <v>5.42</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>0</v>
+        <v>2.32</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>0</v>
+        <v>2.19</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="E39" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="F39" s="24" t="n">
         <v>0</v>
@@ -1690,7 +1690,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="E42" s="24" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="F42" s="24" t="n">
         <v>0</v>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>0</v>
+        <v>3.88</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>0</v>
+        <v>2962.61</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>0</v>
+        <v>51.3</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-63</v>
+        <v>-54</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-25</v>
+        <v>-32</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>0</v>
+        <v>7.32</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-87</v>
+        <v>-84</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=Nonebp [OK]
-HY OAS 5dd=Nonebp
+          <t>HY OAS 20dd=-54.0bp [OK]
+HY OAS 5dd=-2.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-24 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-1</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Flattening</t>
+          <t>Bear Flattening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>18</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.76</v>
+        <v>2.64</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.13</v>
+        <v>4.96</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-17</v>
+        <v>15</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.42</v>
+        <v>5.29</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-13</v>
+        <v>11</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.32</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-54</v>
+        <v>-60</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-32</v>
+        <v>-39</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-22</v>
+        <v>-35</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-54.0bp [OK]
-HY OAS 5dd=-2.0bp
+          <t>HY OAS 20dd=-60.0bp [OK]
+HY OAS 5dd=-17.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-27 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46319</v>
+        <v>46322</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -817,7 +817,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         <v>31</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bear Flattening</t>
+          <t>Bear Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -949,7 +949,7 @@
         <v>64</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-9</v>
+        <v>-4</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -978,7 +978,7 @@
         <v>18</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.64</v>
+        <v>2.66</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.96</v>
+        <v>5</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.29</v>
+        <v>5.33</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1353,7 +1353,7 @@
         <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="F32" s="24" t="n">
         <v>13</v>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.9</v>
+        <v>3.92</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F50" s="24" t="n">
         <v>-10</v>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-60</v>
+        <v>-45</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-39</v>
+        <v>-32</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-60.0bp [OK]
-HY OAS 5dd=-17.0bp
+          <t>HY OAS 20dd=-45.0bp [OK]
+HY OAS 5dd=-7.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-28 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TUE</t>
+          <t>WED</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-7</v>
+        <v>4</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bear Stable</t>
+          <t>Bear Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1038,7 +1038,7 @@
         <v>2.66</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1067,7 +1067,7 @@
         <v>5</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.33</v>
+        <v>5.31</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.21</v>
+        <v>2.25</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.92</v>
+        <v>3.93</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-45</v>
+        <v>-28</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-32</v>
+        <v>-30</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-45.0bp [OK]
-HY OAS 5dd=-7.0bp
+          <t>HY OAS 20dd=-28.0bp [OK]
+HY OAS 5dd=-1.0bp
 HYG 5d=nan% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=nan% [OK]

</xml_diff>

<commit_message>
data: update 2026-10-29 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>WED</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.66</v>
+        <v>2.64</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.31</v>
+        <v>5.3</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.38</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.93</v>
+        <v>3.95</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-28</v>
+        <v>-10</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-30</v>
+        <v>-26</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-28.0bp [OK]
-HY OAS 5dd=-1.0bp
-HYG 5d=nan% [OK]
+          <t>HY OAS 20dd=-10.0bp [OK]
+HY OAS 5dd=15.0bp
+HYG 5d=0.8% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=nan% [OK]
-SPY vs 200MA: above ($SPY=nan, 200MA=nan)
+FXY 5d=0.3% [OK]
+SPY vs 200MA: above ($SPY=772.3099975585938, 200MA=725.2)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-30 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>THU</t>
+          <t>FRI</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>1</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bear Steepening</t>
+          <t>Bear Stable</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.64</v>
+        <v>2.67</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.99</v>
+        <v>5.05</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.3</v>
+        <v>5.37</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.38</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.95</v>
+        <v>3.94</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2962.61</v>
+        <v>2893.77</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>51.3</v>
+        <v>186.95</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-10</v>
+        <v>-2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-26</v>
+        <v>-19</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>7.32</v>
+        <v>7.24</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-84</v>
+        <v>-72</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-10.0bp [OK]
-HY OAS 5dd=15.0bp
-HYG 5d=0.8% [OK]
+          <t>HY OAS 20dd=-2.0bp [OK]
+HY OAS 5dd=13.0bp
+HYG 5d=0.6% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=0.3% [OK]
-SPY vs 200MA: above ($SPY=772.3099975585938, 200MA=725.2)
+FXY 5d=-0.7% [OK]
+SPY vs 200MA: above ($SPY=769.3599853515625, 200MA=725.6)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>

<commit_message>
data: update 2026-10-31 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/template_cleaned_v2.xlsx
+++ b/template_cleaned_v2.xlsx
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B4" s="31" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="28" t="n"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>FRI</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C5" s="28" t="n"/>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>1</v>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>1</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bear Stable</t>
+          <t>Bear Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.67</v>
+        <v>2.63</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5.05</v>
+        <v>4.98</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.37</v>
+        <v>5.32</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>4</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>6</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         <v>3.94</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="F51" s="24" t="n">
         <v>-2</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>-19</v>
+        <v>-12</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E67" s="24" t="n">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>-35</v>
+        <v>-19</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
@@ -2915,11 +2915,11 @@
       <c r="F91" s="21" t="inlineStr">
         <is>
           <t>HY OAS 20dd=-2.0bp [OK]
-HY OAS 5dd=13.0bp
-HYG 5d=0.6% [OK]
+HY OAS 5dd=14.0bp
+HYG 5d=0.5% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=-0.7% [OK]
-SPY vs 200MA: above ($SPY=769.3599853515625, 200MA=725.6)
+FXY 5d=-0.4% [OK]
+SPY vs 200MA: above ($SPY=755.719970703125, 200MA=726.0)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>